<commit_message>
Sistema dinámico: LightGBM ganador + 69 modelos comprimidos
</commit_message>
<xml_diff>
--- a/data/05_modelado/results/resultados_maestro.xlsx
+++ b/data/05_modelado/results/resultados_maestro.xlsx
@@ -545,7 +545,7 @@
         <v>0.7935408590485407</v>
       </c>
       <c r="J2" t="n">
-        <v>16.899</v>
+        <v>4.11</v>
       </c>
       <c r="K2" t="n">
         <v>0.9573</v>
@@ -601,7 +601,7 @@
         <v>0.8611740690867409</v>
       </c>
       <c r="J3" t="n">
-        <v>10.126</v>
+        <v>4.638</v>
       </c>
       <c r="K3" t="n">
         <v>0.9572000000000001</v>
@@ -657,7 +657,7 @@
         <v>0.808414387968506</v>
       </c>
       <c r="J4" t="n">
-        <v>8.996</v>
+        <v>3.96</v>
       </c>
       <c r="K4" t="n">
         <v>0.9560999999999999</v>
@@ -713,7 +713,7 @@
         <v>0.7896000730238919</v>
       </c>
       <c r="J5" t="n">
-        <v>25.148</v>
+        <v>4.562</v>
       </c>
       <c r="K5" t="n">
         <v>0.9564</v>
@@ -769,7 +769,7 @@
         <v>0.8696920960522669</v>
       </c>
       <c r="J6" t="n">
-        <v>16.487</v>
+        <v>4.837</v>
       </c>
       <c r="K6" t="n">
         <v>0.9567</v>
@@ -825,7 +825,7 @@
         <v>0.8072708047410601</v>
       </c>
       <c r="J7" t="n">
-        <v>19.148</v>
+        <v>6.519</v>
       </c>
       <c r="K7" t="n">
         <v>0.9550999999999999</v>
@@ -881,7 +881,7 @@
         <v>0.7965917875586352</v>
       </c>
       <c r="J8" t="n">
-        <v>1442.575</v>
+        <v>525.189</v>
       </c>
       <c r="K8" t="n">
         <v>0.9535</v>
@@ -937,7 +937,7 @@
         <v>0.7965917875586352</v>
       </c>
       <c r="J9" t="n">
-        <v>1390.184</v>
+        <v>2051.132</v>
       </c>
       <c r="K9" t="n">
         <v>0.9535</v>
@@ -993,7 +993,7 @@
         <v>0.8668948124764227</v>
       </c>
       <c r="J10" t="n">
-        <v>34.533</v>
+        <v>9.615</v>
       </c>
       <c r="K10" t="n">
         <v>0.953</v>
@@ -1049,7 +1049,7 @@
         <v>0.7753606564395522</v>
       </c>
       <c r="J11" t="n">
-        <v>27.511</v>
+        <v>10.697</v>
       </c>
       <c r="K11" t="n">
         <v>0.9536</v>
@@ -1105,7 +1105,7 @@
         <v>0.8023123693910341</v>
       </c>
       <c r="J12" t="n">
-        <v>47.524</v>
+        <v>13.366</v>
       </c>
       <c r="K12" t="n">
         <v>0.9519</v>
@@ -1161,7 +1161,7 @@
         <v>0.8312981693136481</v>
       </c>
       <c r="J13" t="n">
-        <v>6342.906</v>
+        <v>1805.924</v>
       </c>
       <c r="K13" t="n">
         <v>0.9514</v>
@@ -1217,7 +1217,7 @@
         <v>0.8285014511882942</v>
       </c>
       <c r="J14" t="n">
-        <v>78.515</v>
+        <v>11.375</v>
       </c>
       <c r="K14" t="n">
         <v>0.95</v>
@@ -1273,7 +1273,7 @@
         <v>0.7579444582216905</v>
       </c>
       <c r="J15" t="n">
-        <v>22.354</v>
+        <v>9.34</v>
       </c>
       <c r="K15" t="n">
         <v>0.9500999999999999</v>
@@ -1329,7 +1329,7 @@
         <v>0.7585815593670509</v>
       </c>
       <c r="J16" t="n">
-        <v>6.195</v>
+        <v>5.683</v>
       </c>
       <c r="K16" t="n">
         <v>0.9530999999999999</v>
@@ -1385,7 +1385,7 @@
         <v>0.7585815593670509</v>
       </c>
       <c r="J17" t="n">
-        <v>6.972</v>
+        <v>8.842000000000001</v>
       </c>
       <c r="K17" t="n">
         <v>0.9530999999999999</v>
@@ -1441,7 +1441,7 @@
         <v>0.841849879357099</v>
       </c>
       <c r="J18" t="n">
-        <v>14.862</v>
+        <v>8.473000000000001</v>
       </c>
       <c r="K18" t="n">
         <v>0.9497</v>
@@ -1497,7 +1497,7 @@
         <v>0.7912527232499509</v>
       </c>
       <c r="J19" t="n">
-        <v>656.528</v>
+        <v>229.459</v>
       </c>
       <c r="K19" t="n">
         <v>0.9483</v>
@@ -1553,7 +1553,7 @@
         <v>0.7912527232499509</v>
       </c>
       <c r="J20" t="n">
-        <v>481.012</v>
+        <v>117.023</v>
       </c>
       <c r="K20" t="n">
         <v>0.9483</v>
@@ -1609,7 +1609,7 @@
         <v>0.8257047330629403</v>
       </c>
       <c r="J21" t="n">
-        <v>1731.173</v>
+        <v>1386.375</v>
       </c>
       <c r="K21" t="n">
         <v>0.9481000000000001</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1665,7 +1665,7 @@
         <v>0.7677332139963536</v>
       </c>
       <c r="J22" t="n">
-        <v>26.029</v>
+        <v>19.913</v>
       </c>
       <c r="K22" t="n">
         <v>0.9489</v>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1721,7 +1721,7 @@
         <v>0.7677332139963536</v>
       </c>
       <c r="J23" t="n">
-        <v>42.487</v>
+        <v>13.523</v>
       </c>
       <c r="K23" t="n">
         <v>0.9489</v>
@@ -1777,7 +1777,7 @@
         <v>0.8105763475291026</v>
       </c>
       <c r="J24" t="n">
-        <v>73.32599999999999</v>
+        <v>25.891</v>
       </c>
       <c r="K24" t="n">
         <v>0.947</v>
@@ -1801,68 +1801,68 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MLP + EBM</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EBM</t>
+          <t>SVM_RBF</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.9379721344826782</v>
+        <v>0.9406270456816881</v>
       </c>
       <c r="E25" t="n">
-        <v>0.003904515896731891</v>
+        <v>0.002782745062362623</v>
       </c>
       <c r="F25" t="n">
-        <v>0.8087287022616166</v>
+        <v>0.8131796087496491</v>
       </c>
       <c r="G25" t="n">
-        <v>0.004188423177670716</v>
+        <v>0.00419568457480829</v>
       </c>
       <c r="H25" t="n">
-        <v>0.8398505034006488</v>
+        <v>0.7714923513771932</v>
       </c>
       <c r="I25" t="n">
-        <v>0.7800661738631012</v>
+        <v>0.8597763562531957</v>
       </c>
       <c r="J25" t="n">
-        <v>1777.304</v>
+        <v>98.999</v>
       </c>
       <c r="K25" t="n">
-        <v>0.9422</v>
+        <v>0.9467</v>
       </c>
       <c r="L25" t="n">
-        <v>0.8099</v>
+        <v>0.8208</v>
       </c>
       <c r="M25" t="n">
-        <v>0.8349</v>
+        <v>0.7706</v>
       </c>
       <c r="N25" t="n">
-        <v>0.7865</v>
+        <v>0.878</v>
       </c>
       <c r="O25" t="n">
-        <v>0.7347</v>
+        <v>0.7397</v>
       </c>
       <c r="P25" t="n">
-        <v>0.2665</v>
+        <v>0.2582</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MLP + EBM</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>SVM_RBF</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1871,43 +1871,43 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.937399108755538</v>
+        <v>0.939318345902185</v>
       </c>
       <c r="E26" t="n">
-        <v>0.005060147566467056</v>
+        <v>0.002834520714023874</v>
       </c>
       <c r="F26" t="n">
-        <v>0.807845391480854</v>
+        <v>0.8154857186662795</v>
       </c>
       <c r="G26" t="n">
-        <v>0.01031190045657124</v>
+        <v>0.005645496372671115</v>
       </c>
       <c r="H26" t="n">
-        <v>0.7955793945456492</v>
+        <v>0.7875058981612502</v>
       </c>
       <c r="I26" t="n">
-        <v>0.8206202022535625</v>
+        <v>0.8456650545942448</v>
       </c>
       <c r="J26" t="n">
-        <v>19.323</v>
+        <v>170.355</v>
       </c>
       <c r="K26" t="n">
-        <v>0.9465</v>
+        <v>0.9458</v>
       </c>
       <c r="L26" t="n">
-        <v>0.8193</v>
+        <v>0.8183</v>
       </c>
       <c r="M26" t="n">
-        <v>0.7984</v>
+        <v>0.7816</v>
       </c>
       <c r="N26" t="n">
-        <v>0.8414</v>
+        <v>0.8587</v>
       </c>
       <c r="O26" t="n">
-        <v>0.7418</v>
+        <v>0.7381</v>
       </c>
       <c r="P26" t="n">
-        <v>0.2923</v>
+        <v>0.2797</v>
       </c>
     </row>
     <row r="27">
@@ -1923,47 +1923,47 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.9373762069707006</v>
+        <v>0.9379721344826782</v>
       </c>
       <c r="E27" t="n">
-        <v>0.002621040993716543</v>
+        <v>0.003904515896731891</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8009504015452423</v>
+        <v>0.8087287022616166</v>
       </c>
       <c r="G27" t="n">
-        <v>0.005202682637965449</v>
+        <v>0.004188423177670716</v>
       </c>
       <c r="H27" t="n">
-        <v>0.8503856976864406</v>
+        <v>0.8398505034006488</v>
       </c>
       <c r="I27" t="n">
-        <v>0.7571827964111664</v>
+        <v>0.7800661738631012</v>
       </c>
       <c r="J27" t="n">
-        <v>428.258</v>
+        <v>512.799</v>
       </c>
       <c r="K27" t="n">
-        <v>0.9421</v>
+        <v>0.9422</v>
       </c>
       <c r="L27" t="n">
-        <v>0.8071</v>
+        <v>0.8099</v>
       </c>
       <c r="M27" t="n">
-        <v>0.8478</v>
+        <v>0.8349</v>
       </c>
       <c r="N27" t="n">
-        <v>0.7702</v>
+        <v>0.7865</v>
       </c>
       <c r="O27" t="n">
-        <v>0.7327</v>
+        <v>0.7347</v>
       </c>
       <c r="P27" t="n">
-        <v>0.2654</v>
+        <v>0.2665</v>
       </c>
     </row>
     <row r="28">
@@ -1974,388 +1974,388 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EBM</t>
+          <t>MLP</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.9373762069707006</v>
+        <v>0.937399108755538</v>
       </c>
       <c r="E28" t="n">
-        <v>0.002621040993716543</v>
+        <v>0.005060147566467056</v>
       </c>
       <c r="F28" t="n">
-        <v>0.8009504015452423</v>
+        <v>0.807845391480854</v>
       </c>
       <c r="G28" t="n">
-        <v>0.005202682637965449</v>
+        <v>0.01031190045657124</v>
       </c>
       <c r="H28" t="n">
-        <v>0.8503856976864406</v>
+        <v>0.7955793945456492</v>
       </c>
       <c r="I28" t="n">
-        <v>0.7571827964111664</v>
+        <v>0.8206202022535625</v>
       </c>
       <c r="J28" t="n">
-        <v>280.69</v>
+        <v>23.548</v>
       </c>
       <c r="K28" t="n">
-        <v>0.9421</v>
+        <v>0.9465</v>
       </c>
       <c r="L28" t="n">
-        <v>0.8071</v>
+        <v>0.8193</v>
       </c>
       <c r="M28" t="n">
-        <v>0.8478</v>
+        <v>0.7984</v>
       </c>
       <c r="N28" t="n">
-        <v>0.7702</v>
+        <v>0.8414</v>
       </c>
       <c r="O28" t="n">
-        <v>0.7327</v>
+        <v>0.7418</v>
       </c>
       <c r="P28" t="n">
-        <v>0.2654</v>
+        <v>0.2923</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>MLP + EBM</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>EBM</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.9315129619923168</v>
+        <v>0.9373762069707006</v>
       </c>
       <c r="E29" t="n">
-        <v>0.00376073451208329</v>
+        <v>0.002621040993716543</v>
       </c>
       <c r="F29" t="n">
-        <v>0.7591554666450639</v>
+        <v>0.8009504015452423</v>
       </c>
       <c r="G29" t="n">
-        <v>0.006986982179453731</v>
+        <v>0.005202682637965449</v>
       </c>
       <c r="H29" t="n">
-        <v>0.8768327532554583</v>
+        <v>0.8503856976864406</v>
       </c>
       <c r="I29" t="n">
-        <v>0.6695891840630204</v>
+        <v>0.7571827964111664</v>
       </c>
       <c r="J29" t="n">
-        <v>35.522</v>
+        <v>231.967</v>
       </c>
       <c r="K29" t="n">
-        <v>0.9336</v>
+        <v>0.9421</v>
       </c>
       <c r="L29" t="n">
-        <v>0.761</v>
+        <v>0.8071</v>
       </c>
       <c r="M29" t="n">
-        <v>0.8643</v>
+        <v>0.8478</v>
       </c>
       <c r="N29" t="n">
-        <v>0.6797</v>
+        <v>0.7702</v>
       </c>
       <c r="O29" t="n">
-        <v>0.678</v>
+        <v>0.7327</v>
       </c>
       <c r="P29" t="n">
-        <v>0.3122</v>
+        <v>0.2654</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>MLP + EBM</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>EBM</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.9313679768742575</v>
+        <v>0.9373762069707006</v>
       </c>
       <c r="E30" t="n">
-        <v>0.003516553961544682</v>
+        <v>0.002621040993716543</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7810657033018569</v>
+        <v>0.8009504015452423</v>
       </c>
       <c r="G30" t="n">
-        <v>0.007559627176103657</v>
+        <v>0.005202682637965449</v>
       </c>
       <c r="H30" t="n">
-        <v>0.7330423223469913</v>
+        <v>0.8503856976864406</v>
       </c>
       <c r="I30" t="n">
-        <v>0.836002959729424</v>
+        <v>0.7571827964111664</v>
       </c>
       <c r="J30" t="n">
-        <v>2.793</v>
+        <v>205.061</v>
       </c>
       <c r="K30" t="n">
-        <v>0.9343</v>
+        <v>0.9421</v>
       </c>
       <c r="L30" t="n">
-        <v>0.7828000000000001</v>
+        <v>0.8071</v>
       </c>
       <c r="M30" t="n">
-        <v>0.7221</v>
+        <v>0.8478</v>
       </c>
       <c r="N30" t="n">
-        <v>0.8546</v>
+        <v>0.7702</v>
       </c>
       <c r="O30" t="n">
-        <v>0.6819</v>
+        <v>0.7327</v>
       </c>
       <c r="P30" t="n">
-        <v>0.3506</v>
+        <v>0.2654</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>SVM_RBF</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.9308044637766206</v>
+        <v>0.9359077674488931</v>
       </c>
       <c r="E31" t="n">
-        <v>0.003272936094553819</v>
+        <v>0.002933434465342158</v>
       </c>
       <c r="F31" t="n">
-        <v>0.783444623490177</v>
+        <v>0.8098878515300243</v>
       </c>
       <c r="G31" t="n">
-        <v>0.009242881824032642</v>
+        <v>0.001438437931955519</v>
       </c>
       <c r="H31" t="n">
-        <v>0.7465855429302748</v>
+        <v>0.871526206690789</v>
       </c>
       <c r="I31" t="n">
-        <v>0.8243067778934707</v>
+        <v>0.7565469877240699</v>
       </c>
       <c r="J31" t="n">
-        <v>34.249</v>
+        <v>80.964</v>
       </c>
       <c r="K31" t="n">
-        <v>0.9332</v>
+        <v>0.9428</v>
       </c>
       <c r="L31" t="n">
-        <v>0.785</v>
+        <v>0.8158</v>
       </c>
       <c r="M31" t="n">
-        <v>0.7346</v>
+        <v>0.8703</v>
       </c>
       <c r="N31" t="n">
-        <v>0.8429</v>
+        <v>0.7677</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6873</v>
+        <v>0.7462</v>
       </c>
       <c r="P31" t="n">
-        <v>0.3451</v>
+        <v>0.2597</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.9298593588287318</v>
+        <v>0.9315129619923168</v>
       </c>
       <c r="E32" t="n">
-        <v>0.002940966150935203</v>
+        <v>0.00376073451208329</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7857642160266411</v>
+        <v>0.7591554666450639</v>
       </c>
       <c r="G32" t="n">
-        <v>0.007518361017691409</v>
+        <v>0.006986982179453731</v>
       </c>
       <c r="H32" t="n">
-        <v>0.7545141466774683</v>
+        <v>0.8768327532554583</v>
       </c>
       <c r="I32" t="n">
-        <v>0.8201101659112517</v>
+        <v>0.6695891840630204</v>
       </c>
       <c r="J32" t="n">
-        <v>71.434</v>
+        <v>3.791</v>
       </c>
       <c r="K32" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.9336</v>
       </c>
       <c r="L32" t="n">
-        <v>0.7861</v>
+        <v>0.761</v>
       </c>
       <c r="M32" t="n">
-        <v>0.7417</v>
+        <v>0.8643</v>
       </c>
       <c r="N32" t="n">
-        <v>0.8363</v>
+        <v>0.6797</v>
       </c>
       <c r="O32" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.678</v>
       </c>
       <c r="P32" t="n">
-        <v>0.445</v>
+        <v>0.3122</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Bagging</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.9282010462024315</v>
+        <v>0.9313679768742575</v>
       </c>
       <c r="E33" t="n">
-        <v>0.003252072683053184</v>
+        <v>0.003516553961544682</v>
       </c>
       <c r="F33" t="n">
-        <v>0.7680192654030435</v>
+        <v>0.7810657033018569</v>
       </c>
       <c r="G33" t="n">
-        <v>0.01137668644677119</v>
+        <v>0.007559627176103657</v>
       </c>
       <c r="H33" t="n">
-        <v>0.830378849828832</v>
+        <v>0.7330423223469913</v>
       </c>
       <c r="I33" t="n">
-        <v>0.7151064945219965</v>
+        <v>0.836002959729424</v>
       </c>
       <c r="J33" t="n">
-        <v>20.731</v>
+        <v>3.808</v>
       </c>
       <c r="K33" t="n">
-        <v>0.9339</v>
+        <v>0.9343</v>
       </c>
       <c r="L33" t="n">
-        <v>0.7713</v>
+        <v>0.7828000000000001</v>
       </c>
       <c r="M33" t="n">
-        <v>0.8138</v>
+        <v>0.7221</v>
       </c>
       <c r="N33" t="n">
-        <v>0.7331</v>
+        <v>0.8546</v>
       </c>
       <c r="O33" t="n">
-        <v>0.6836</v>
+        <v>0.6819</v>
       </c>
       <c r="P33" t="n">
-        <v>0.2924</v>
+        <v>0.3506</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bagging</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.9282010462024315</v>
+        <v>0.9308044637766206</v>
       </c>
       <c r="E34" t="n">
-        <v>0.003252072683053184</v>
+        <v>0.003272936094553819</v>
       </c>
       <c r="F34" t="n">
-        <v>0.7680192654030435</v>
+        <v>0.783444623490177</v>
       </c>
       <c r="G34" t="n">
-        <v>0.01137668644677119</v>
+        <v>0.009242881824032642</v>
       </c>
       <c r="H34" t="n">
-        <v>0.830378849828832</v>
+        <v>0.7465855429302748</v>
       </c>
       <c r="I34" t="n">
-        <v>0.7151064945219965</v>
+        <v>0.8243067778934707</v>
       </c>
       <c r="J34" t="n">
-        <v>18.024</v>
+        <v>5.966</v>
       </c>
       <c r="K34" t="n">
-        <v>0.9339</v>
+        <v>0.9332</v>
       </c>
       <c r="L34" t="n">
-        <v>0.7713</v>
+        <v>0.785</v>
       </c>
       <c r="M34" t="n">
-        <v>0.8138</v>
+        <v>0.7346</v>
       </c>
       <c r="N34" t="n">
-        <v>0.7331</v>
+        <v>0.8429</v>
       </c>
       <c r="O34" t="n">
-        <v>0.6836</v>
+        <v>0.6873</v>
       </c>
       <c r="P34" t="n">
-        <v>0.2924</v>
+        <v>0.3451</v>
       </c>
     </row>
     <row r="35">
@@ -2371,47 +2371,47 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.9240837379510936</v>
+        <v>0.9298593588287318</v>
       </c>
       <c r="E35" t="n">
-        <v>0.003312467116935505</v>
+        <v>0.002940966150935203</v>
       </c>
       <c r="F35" t="n">
-        <v>0.7531045823849295</v>
+        <v>0.7857642160266411</v>
       </c>
       <c r="G35" t="n">
-        <v>0.007630946081345134</v>
+        <v>0.007518361017691409</v>
       </c>
       <c r="H35" t="n">
-        <v>0.8313178176975002</v>
+        <v>0.7545141466774683</v>
       </c>
       <c r="I35" t="n">
-        <v>0.6885311292611743</v>
+        <v>0.8201101659112517</v>
       </c>
       <c r="J35" t="n">
-        <v>31.611</v>
+        <v>15.005</v>
       </c>
       <c r="K35" t="n">
-        <v>0.9301</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="L35" t="n">
-        <v>0.7606000000000001</v>
+        <v>0.7861</v>
       </c>
       <c r="M35" t="n">
-        <v>0.8269</v>
+        <v>0.7417</v>
       </c>
       <c r="N35" t="n">
-        <v>0.7040999999999999</v>
+        <v>0.8363</v>
       </c>
       <c r="O35" t="n">
-        <v>0.6724</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P35" t="n">
-        <v>0.4058</v>
+        <v>0.445</v>
       </c>
     </row>
     <row r="36">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>Bagging</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2431,43 +2431,43 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.9240837379510936</v>
+        <v>0.9282010462024315</v>
       </c>
       <c r="E36" t="n">
-        <v>0.003312467116935505</v>
+        <v>0.003252072683053184</v>
       </c>
       <c r="F36" t="n">
-        <v>0.7531045823849295</v>
+        <v>0.7680192654030435</v>
       </c>
       <c r="G36" t="n">
-        <v>0.007630946081345134</v>
+        <v>0.01137668644677119</v>
       </c>
       <c r="H36" t="n">
-        <v>0.8313178176975002</v>
+        <v>0.830378849828832</v>
       </c>
       <c r="I36" t="n">
-        <v>0.6885311292611743</v>
+        <v>0.7151064945219965</v>
       </c>
       <c r="J36" t="n">
-        <v>33.396</v>
+        <v>2.148</v>
       </c>
       <c r="K36" t="n">
-        <v>0.9301</v>
+        <v>0.9339</v>
       </c>
       <c r="L36" t="n">
-        <v>0.7606000000000001</v>
+        <v>0.7713</v>
       </c>
       <c r="M36" t="n">
-        <v>0.8269</v>
+        <v>0.8138</v>
       </c>
       <c r="N36" t="n">
-        <v>0.7040999999999999</v>
+        <v>0.7331</v>
       </c>
       <c r="O36" t="n">
-        <v>0.6724</v>
+        <v>0.6836</v>
       </c>
       <c r="P36" t="n">
-        <v>0.4058</v>
+        <v>0.2924</v>
       </c>
     </row>
     <row r="37">
@@ -2483,170 +2483,170 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.9239479055348996</v>
+        <v>0.9282010462024315</v>
       </c>
       <c r="E37" t="n">
-        <v>0.001883537286232897</v>
+        <v>0.003252072683053184</v>
       </c>
       <c r="F37" t="n">
-        <v>0.7685357021647838</v>
+        <v>0.7680192654030435</v>
       </c>
       <c r="G37" t="n">
-        <v>0.004666734889156638</v>
+        <v>0.01137668644677119</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7118950317075459</v>
+        <v>0.830378849828832</v>
       </c>
       <c r="I37" t="n">
-        <v>0.8353645661257998</v>
+        <v>0.7151064945219965</v>
       </c>
       <c r="J37" t="n">
-        <v>35.549</v>
+        <v>5.371</v>
       </c>
       <c r="K37" t="n">
-        <v>0.93</v>
+        <v>0.9339</v>
       </c>
       <c r="L37" t="n">
-        <v>0.7708</v>
+        <v>0.7713</v>
       </c>
       <c r="M37" t="n">
-        <v>0.7163</v>
+        <v>0.8138</v>
       </c>
       <c r="N37" t="n">
-        <v>0.8343</v>
+        <v>0.7331</v>
       </c>
       <c r="O37" t="n">
-        <v>0.6655</v>
+        <v>0.6836</v>
       </c>
       <c r="P37" t="n">
-        <v>0.3238</v>
+        <v>0.2924</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.9205603346469882</v>
+        <v>0.9240837379510936</v>
       </c>
       <c r="E38" t="n">
-        <v>0.003541831237419791</v>
+        <v>0.003312467116935505</v>
       </c>
       <c r="F38" t="n">
-        <v>0.7755728698719533</v>
+        <v>0.7531045823849295</v>
       </c>
       <c r="G38" t="n">
-        <v>0.005642045979370998</v>
+        <v>0.007630946081345134</v>
       </c>
       <c r="H38" t="n">
-        <v>0.8330307606902737</v>
+        <v>0.8313178176975002</v>
       </c>
       <c r="I38" t="n">
-        <v>0.7256528731751095</v>
+        <v>0.6885311292611743</v>
       </c>
       <c r="J38" t="n">
-        <v>6.912</v>
+        <v>6.983</v>
       </c>
       <c r="K38" t="n">
-        <v>0.9273</v>
+        <v>0.9301</v>
       </c>
       <c r="L38" t="n">
-        <v>0.7784</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>0.8207</v>
+        <v>0.8269</v>
       </c>
       <c r="N38" t="n">
-        <v>0.7402</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="O38" t="n">
-        <v>0.6933</v>
+        <v>0.6724</v>
       </c>
       <c r="P38" t="n">
-        <v>0.6479</v>
+        <v>0.4058</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.9205603346469882</v>
+        <v>0.9240837379510936</v>
       </c>
       <c r="E39" t="n">
-        <v>0.003541831237419791</v>
+        <v>0.003312467116935505</v>
       </c>
       <c r="F39" t="n">
-        <v>0.7755728698719533</v>
+        <v>0.7531045823849295</v>
       </c>
       <c r="G39" t="n">
-        <v>0.005642045979370998</v>
+        <v>0.007630946081345134</v>
       </c>
       <c r="H39" t="n">
-        <v>0.8330307606902737</v>
+        <v>0.8313178176975002</v>
       </c>
       <c r="I39" t="n">
-        <v>0.7256528731751095</v>
+        <v>0.6885311292611743</v>
       </c>
       <c r="J39" t="n">
-        <v>5.686</v>
+        <v>7.129</v>
       </c>
       <c r="K39" t="n">
-        <v>0.9273</v>
+        <v>0.9301</v>
       </c>
       <c r="L39" t="n">
-        <v>0.7784</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>0.8207</v>
+        <v>0.8269</v>
       </c>
       <c r="N39" t="n">
-        <v>0.7402</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>0.6933</v>
+        <v>0.6724</v>
       </c>
       <c r="P39" t="n">
-        <v>0.6479</v>
+        <v>0.4058</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>Bagging</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2655,110 +2655,110 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.9165453449080809</v>
+        <v>0.9239479055348996</v>
       </c>
       <c r="E40" t="n">
-        <v>0.002630592056380005</v>
+        <v>0.001883537286232897</v>
       </c>
       <c r="F40" t="n">
-        <v>0.7610276129677098</v>
+        <v>0.7685357021647838</v>
       </c>
       <c r="G40" t="n">
-        <v>0.003930919350853034</v>
+        <v>0.004666734889156638</v>
       </c>
       <c r="H40" t="n">
-        <v>0.6887434653302952</v>
+        <v>0.7118950317075459</v>
       </c>
       <c r="I40" t="n">
-        <v>0.8503684717731155</v>
+        <v>0.8353645661257998</v>
       </c>
       <c r="J40" t="n">
-        <v>13.685</v>
+        <v>3.993</v>
       </c>
       <c r="K40" t="n">
-        <v>0.9235</v>
+        <v>0.93</v>
       </c>
       <c r="L40" t="n">
-        <v>0.7678</v>
+        <v>0.7708</v>
       </c>
       <c r="M40" t="n">
-        <v>0.6908</v>
+        <v>0.7163</v>
       </c>
       <c r="N40" t="n">
-        <v>0.8643</v>
+        <v>0.8343</v>
       </c>
       <c r="O40" t="n">
-        <v>0.656</v>
+        <v>0.6655</v>
       </c>
       <c r="P40" t="n">
-        <v>0.9113</v>
+        <v>0.3238</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SGDElasticNet</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.9080340040199995</v>
+        <v>0.9205603346469882</v>
       </c>
       <c r="E41" t="n">
-        <v>0.003540900512979701</v>
+        <v>0.003541831237419791</v>
       </c>
       <c r="F41" t="n">
-        <v>0.7498507807360217</v>
+        <v>0.7755728698719533</v>
       </c>
       <c r="G41" t="n">
-        <v>0.006027893023129959</v>
+        <v>0.005642045979370998</v>
       </c>
       <c r="H41" t="n">
-        <v>0.6816717829089194</v>
+        <v>0.8330307606902737</v>
       </c>
       <c r="I41" t="n">
-        <v>0.8333322562847802</v>
+        <v>0.7256528731751095</v>
       </c>
       <c r="J41" t="n">
-        <v>4.623</v>
+        <v>3.299</v>
       </c>
       <c r="K41" t="n">
-        <v>0.9134</v>
+        <v>0.9273</v>
       </c>
       <c r="L41" t="n">
-        <v>0.755</v>
+        <v>0.7784</v>
       </c>
       <c r="M41" t="n">
-        <v>0.6817</v>
+        <v>0.8207</v>
       </c>
       <c r="N41" t="n">
-        <v>0.846</v>
+        <v>0.7402</v>
       </c>
       <c r="O41" t="n">
-        <v>0.6375999999999999</v>
+        <v>0.6933</v>
       </c>
       <c r="P41" t="n">
-        <v>0.383</v>
+        <v>0.6479</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SGDElasticNet</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2767,54 +2767,54 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.9058661087149359</v>
+        <v>0.9205603346469882</v>
       </c>
       <c r="E42" t="n">
-        <v>0.004884769542416435</v>
+        <v>0.003541831237419791</v>
       </c>
       <c r="F42" t="n">
-        <v>0.747327937025999</v>
+        <v>0.7755728698719533</v>
       </c>
       <c r="G42" t="n">
-        <v>0.01376937941294494</v>
+        <v>0.005642045979370998</v>
       </c>
       <c r="H42" t="n">
-        <v>0.6852618333117529</v>
+        <v>0.8330307606902737</v>
       </c>
       <c r="I42" t="n">
-        <v>0.8231616598718366</v>
+        <v>0.7256528731751095</v>
       </c>
       <c r="J42" t="n">
-        <v>0.764</v>
+        <v>4.374</v>
       </c>
       <c r="K42" t="n">
-        <v>0.9132</v>
+        <v>0.9273</v>
       </c>
       <c r="L42" t="n">
-        <v>0.7605</v>
+        <v>0.7784</v>
       </c>
       <c r="M42" t="n">
-        <v>0.7102000000000001</v>
+        <v>0.8207</v>
       </c>
       <c r="N42" t="n">
-        <v>0.8185</v>
+        <v>0.7402</v>
       </c>
       <c r="O42" t="n">
-        <v>0.6513</v>
+        <v>0.6933</v>
       </c>
       <c r="P42" t="n">
-        <v>0.3624</v>
+        <v>0.6479</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2823,43 +2823,43 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.9057562632928381</v>
+        <v>0.9165453449080809</v>
       </c>
       <c r="E43" t="n">
-        <v>0.003212375345637456</v>
+        <v>0.002630592056380005</v>
       </c>
       <c r="F43" t="n">
-        <v>0.7493470312335072</v>
+        <v>0.7610276129677098</v>
       </c>
       <c r="G43" t="n">
-        <v>0.006349929513041751</v>
+        <v>0.003930919350853034</v>
       </c>
       <c r="H43" t="n">
-        <v>0.6980245716132399</v>
+        <v>0.6887434653302952</v>
       </c>
       <c r="I43" t="n">
-        <v>0.8090520545643567</v>
+        <v>0.8503684717731155</v>
       </c>
       <c r="J43" t="n">
-        <v>16.298</v>
+        <v>7.661</v>
       </c>
       <c r="K43" t="n">
-        <v>0.9072</v>
+        <v>0.9235</v>
       </c>
       <c r="L43" t="n">
-        <v>0.7613</v>
+        <v>0.7678</v>
       </c>
       <c r="M43" t="n">
-        <v>0.7294</v>
+        <v>0.6908</v>
       </c>
       <c r="N43" t="n">
-        <v>0.7961</v>
+        <v>0.8643</v>
       </c>
       <c r="O43" t="n">
-        <v>0.6564</v>
+        <v>0.656</v>
       </c>
       <c r="P43" t="n">
-        <v>0.3845</v>
+        <v>0.9113</v>
       </c>
     </row>
     <row r="44">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SVM_RBF</t>
+          <t>LogReg</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2879,43 +2879,43 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.9055556282596344</v>
+        <v>0.9109499135777416</v>
       </c>
       <c r="E44" t="n">
-        <v>0.003415658412659005</v>
+        <v>0.004286400054514685</v>
       </c>
       <c r="F44" t="n">
-        <v>0.7564983454614655</v>
+        <v>0.7550972149437635</v>
       </c>
       <c r="G44" t="n">
-        <v>0.006123515596986275</v>
+        <v>0.006871686473038936</v>
       </c>
       <c r="H44" t="n">
-        <v>0.7119822164425902</v>
+        <v>0.6875271951410917</v>
       </c>
       <c r="I44" t="n">
-        <v>0.8071431744875202</v>
+        <v>0.8376554483981998</v>
       </c>
       <c r="J44" t="n">
-        <v>112.901</v>
+        <v>1.926</v>
       </c>
       <c r="K44" t="n">
-        <v>0.9142</v>
+        <v>0.9161</v>
       </c>
       <c r="L44" t="n">
-        <v>0.7623</v>
+        <v>0.7601</v>
       </c>
       <c r="M44" t="n">
-        <v>0.7079</v>
+        <v>0.6881</v>
       </c>
       <c r="N44" t="n">
-        <v>0.8256</v>
+        <v>0.849</v>
       </c>
       <c r="O44" t="n">
-        <v>0.653</v>
+        <v>0.6456</v>
       </c>
       <c r="P44" t="n">
-        <v>0.3252</v>
+        <v>0.3731</v>
       </c>
     </row>
     <row r="45">
@@ -2926,52 +2926,52 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SGDElasticNet</t>
+          <t>LogReg</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.9051599001258989</v>
+        <v>0.9105889776283842</v>
       </c>
       <c r="E45" t="n">
-        <v>0.003946958430842508</v>
+        <v>0.004398031409553485</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7393836496871475</v>
+        <v>0.7554974623059211</v>
       </c>
       <c r="G45" t="n">
-        <v>0.007832908049006399</v>
+        <v>0.007898496562435691</v>
       </c>
       <c r="H45" t="n">
-        <v>0.7825349652936302</v>
+        <v>0.691385867513496</v>
       </c>
       <c r="I45" t="n">
-        <v>0.7017556429939472</v>
+        <v>0.8329515465474806</v>
       </c>
       <c r="J45" t="n">
-        <v>0.822</v>
+        <v>3.339</v>
       </c>
       <c r="K45" t="n">
-        <v>0.9069</v>
+        <v>0.9157999999999999</v>
       </c>
       <c r="L45" t="n">
-        <v>0.7494</v>
+        <v>0.7614</v>
       </c>
       <c r="M45" t="n">
-        <v>0.8022</v>
+        <v>0.6926</v>
       </c>
       <c r="N45" t="n">
-        <v>0.7030999999999999</v>
+        <v>0.8454</v>
       </c>
       <c r="O45" t="n">
-        <v>0.6552</v>
+        <v>0.6484</v>
       </c>
       <c r="P45" t="n">
-        <v>0.3398</v>
+        <v>0.3696</v>
       </c>
     </row>
     <row r="46">
@@ -2982,52 +2982,52 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>LogReg</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.9038660096861791</v>
+        <v>0.9103383330709626</v>
       </c>
       <c r="E46" t="n">
-        <v>0.00580205681122376</v>
+        <v>0.004736296862742382</v>
       </c>
       <c r="F46" t="n">
-        <v>0.7359116552775953</v>
+        <v>0.7490915130761712</v>
       </c>
       <c r="G46" t="n">
-        <v>0.007200138561096124</v>
+        <v>0.004167737120005451</v>
       </c>
       <c r="H46" t="n">
-        <v>0.6491643590957055</v>
+        <v>0.7927372623217182</v>
       </c>
       <c r="I46" t="n">
-        <v>0.849860858790049</v>
+        <v>0.7105256185422525</v>
       </c>
       <c r="J46" t="n">
-        <v>3.093</v>
+        <v>3.013</v>
       </c>
       <c r="K46" t="n">
-        <v>0.9001</v>
+        <v>0.9153</v>
       </c>
       <c r="L46" t="n">
-        <v>0.7337</v>
+        <v>0.7577</v>
       </c>
       <c r="M46" t="n">
-        <v>0.6777</v>
+        <v>0.7899</v>
       </c>
       <c r="N46" t="n">
-        <v>0.7997</v>
+        <v>0.728</v>
       </c>
       <c r="O46" t="n">
-        <v>0.6103</v>
+        <v>0.6632</v>
       </c>
       <c r="P46" t="n">
-        <v>0.6812</v>
+        <v>0.3263</v>
       </c>
     </row>
     <row r="47">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SVM_RBF</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3047,99 +3047,99 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.9032101966333258</v>
+        <v>0.90952151997194</v>
       </c>
       <c r="E47" t="n">
-        <v>0.00242878605028493</v>
+        <v>0.003815404540050895</v>
       </c>
       <c r="F47" t="n">
-        <v>0.7582709660512823</v>
+        <v>0.7529516133446159</v>
       </c>
       <c r="G47" t="n">
-        <v>0.004171604488190237</v>
+        <v>0.005847307384366608</v>
       </c>
       <c r="H47" t="n">
-        <v>0.7225322042312822</v>
+        <v>0.6856266400359575</v>
       </c>
       <c r="I47" t="n">
-        <v>0.7979907928504441</v>
+        <v>0.8351127791003036</v>
       </c>
       <c r="J47" t="n">
-        <v>448.563</v>
+        <v>0.87</v>
       </c>
       <c r="K47" t="n">
-        <v>0.9126</v>
+        <v>0.9146</v>
       </c>
       <c r="L47" t="n">
-        <v>0.7613</v>
+        <v>0.7565</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7163</v>
+        <v>0.6832</v>
       </c>
       <c r="N47" t="n">
-        <v>0.8124</v>
+        <v>0.8475</v>
       </c>
       <c r="O47" t="n">
-        <v>0.6536</v>
+        <v>0.6399</v>
       </c>
       <c r="P47" t="n">
-        <v>0.357</v>
+        <v>0.3826</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>SVM_lineal</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.9026765293335541</v>
+        <v>0.9081345416562769</v>
       </c>
       <c r="E48" t="n">
-        <v>0.004878767896935301</v>
+        <v>0.004032424685030564</v>
       </c>
       <c r="F48" t="n">
-        <v>0.7361697829446927</v>
+        <v>0.7566461040751585</v>
       </c>
       <c r="G48" t="n">
-        <v>0.01112601087569545</v>
+        <v>0.006902453984135339</v>
       </c>
       <c r="H48" t="n">
-        <v>0.7754078384204025</v>
+        <v>0.696688403837072</v>
       </c>
       <c r="I48" t="n">
-        <v>0.7015024827315458</v>
+        <v>0.8281202567791455</v>
       </c>
       <c r="J48" t="n">
-        <v>2.588</v>
+        <v>146.073</v>
       </c>
       <c r="K48" t="n">
-        <v>0.9109</v>
+        <v>0.9144</v>
       </c>
       <c r="L48" t="n">
-        <v>0.7374000000000001</v>
+        <v>0.7634</v>
       </c>
       <c r="M48" t="n">
-        <v>0.8228</v>
+        <v>0.6969</v>
       </c>
       <c r="N48" t="n">
-        <v>0.668</v>
+        <v>0.8439</v>
       </c>
       <c r="O48" t="n">
-        <v>0.6441</v>
+        <v>0.6518</v>
       </c>
       <c r="P48" t="n">
-        <v>0.373</v>
+        <v>0.3747</v>
       </c>
     </row>
     <row r="49">
@@ -3150,63 +3150,63 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SVM_RBF</t>
+          <t>SGDElasticNet</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.9000351655149885</v>
+        <v>0.9080340040199995</v>
       </c>
       <c r="E49" t="n">
-        <v>0.00386559300205514</v>
+        <v>0.003540900512979701</v>
       </c>
       <c r="F49" t="n">
-        <v>0.7400158105610716</v>
+        <v>0.7498507807360217</v>
       </c>
       <c r="G49" t="n">
-        <v>0.001999545657618309</v>
+        <v>0.006027893023129959</v>
       </c>
       <c r="H49" t="n">
-        <v>0.8241293282827232</v>
+        <v>0.6816717829089194</v>
       </c>
       <c r="I49" t="n">
-        <v>0.6716241595992087</v>
+        <v>0.8333322562847802</v>
       </c>
       <c r="J49" t="n">
-        <v>109.93</v>
+        <v>1.206</v>
       </c>
       <c r="K49" t="n">
-        <v>0.9083</v>
+        <v>0.9134</v>
       </c>
       <c r="L49" t="n">
-        <v>0.7541</v>
+        <v>0.755</v>
       </c>
       <c r="M49" t="n">
-        <v>0.8293</v>
+        <v>0.6817</v>
       </c>
       <c r="N49" t="n">
-        <v>0.6914</v>
+        <v>0.846</v>
       </c>
       <c r="O49" t="n">
-        <v>0.665</v>
+        <v>0.6375999999999999</v>
       </c>
       <c r="P49" t="n">
-        <v>0.3283</v>
+        <v>0.383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>SVM_lineal</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3215,43 +3215,43 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.8999538184092056</v>
+        <v>0.9078242602398875</v>
       </c>
       <c r="E50" t="n">
-        <v>0.003311414395632856</v>
+        <v>0.003887058137010558</v>
       </c>
       <c r="F50" t="n">
-        <v>0.7329380126007593</v>
+        <v>0.7552133614589875</v>
       </c>
       <c r="G50" t="n">
-        <v>0.009663686372255531</v>
+        <v>0.007235999710313818</v>
       </c>
       <c r="H50" t="n">
-        <v>0.6545947385865329</v>
+        <v>0.6925465999302066</v>
       </c>
       <c r="I50" t="n">
-        <v>0.8347279496522884</v>
+        <v>0.8305362651671997</v>
       </c>
       <c r="J50" t="n">
-        <v>2.813</v>
+        <v>75.029</v>
       </c>
       <c r="K50" t="n">
-        <v>0.9133</v>
+        <v>0.914</v>
       </c>
       <c r="L50" t="n">
-        <v>0.7453</v>
+        <v>0.7624</v>
       </c>
       <c r="M50" t="n">
-        <v>0.6617</v>
+        <v>0.6918</v>
       </c>
       <c r="N50" t="n">
-        <v>0.8531</v>
+        <v>0.849</v>
       </c>
       <c r="O50" t="n">
-        <v>0.6201</v>
+        <v>0.6494</v>
       </c>
       <c r="P50" t="n">
-        <v>0.4213</v>
+        <v>0.332</v>
       </c>
     </row>
     <row r="51">
@@ -3262,52 +3262,52 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.8997149781030049</v>
+        <v>0.9072716669671005</v>
       </c>
       <c r="E51" t="n">
-        <v>0.004231156829102635</v>
+        <v>0.004042803272633883</v>
       </c>
       <c r="F51" t="n">
-        <v>0.7267192283247618</v>
+        <v>0.7454656595468206</v>
       </c>
       <c r="G51" t="n">
-        <v>0.01577460752560449</v>
+        <v>0.003291535615744811</v>
       </c>
       <c r="H51" t="n">
-        <v>0.7864884931006975</v>
+        <v>0.7862751778567668</v>
       </c>
       <c r="I51" t="n">
-        <v>0.6805268544554671</v>
+        <v>0.7091274210368586</v>
       </c>
       <c r="J51" t="n">
-        <v>18.532</v>
+        <v>1.663</v>
       </c>
       <c r="K51" t="n">
-        <v>0.8977000000000001</v>
+        <v>0.912</v>
       </c>
       <c r="L51" t="n">
-        <v>0.7271</v>
+        <v>0.7466</v>
       </c>
       <c r="M51" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7783</v>
       </c>
       <c r="N51" t="n">
-        <v>0.6914</v>
+        <v>0.7173</v>
       </c>
       <c r="O51" t="n">
-        <v>0.6223</v>
+        <v>0.6477000000000001</v>
       </c>
       <c r="P51" t="n">
-        <v>0.7409</v>
+        <v>0.3371</v>
       </c>
     </row>
     <row r="52">
@@ -3318,52 +3318,52 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.8904495092967712</v>
+        <v>0.9072716669671005</v>
       </c>
       <c r="E52" t="n">
-        <v>0.0127432871352812</v>
+        <v>0.004042803272633883</v>
       </c>
       <c r="F52" t="n">
-        <v>0.7261581011517647</v>
+        <v>0.7454656595468206</v>
       </c>
       <c r="G52" t="n">
-        <v>0.01875638316318416</v>
+        <v>0.003291535615744811</v>
       </c>
       <c r="H52" t="n">
-        <v>0.6575439998429703</v>
+        <v>0.7862751778567668</v>
       </c>
       <c r="I52" t="n">
-        <v>0.8189757914489345</v>
+        <v>0.7091274210368586</v>
       </c>
       <c r="J52" t="n">
-        <v>2.54</v>
+        <v>2.364</v>
       </c>
       <c r="K52" t="n">
-        <v>0.8931</v>
+        <v>0.912</v>
       </c>
       <c r="L52" t="n">
-        <v>0.7156</v>
+        <v>0.7466</v>
       </c>
       <c r="M52" t="n">
-        <v>0.6206</v>
+        <v>0.7783</v>
       </c>
       <c r="N52" t="n">
-        <v>0.8449</v>
+        <v>0.7173</v>
       </c>
       <c r="O52" t="n">
-        <v>0.5709</v>
+        <v>0.6477000000000001</v>
       </c>
       <c r="P52" t="n">
-        <v>0.8991</v>
+        <v>0.3371</v>
       </c>
     </row>
     <row r="53">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LogReg</t>
+          <t>SGDElasticNet</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3383,54 +3383,54 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.8850984813019854</v>
+        <v>0.9058661087149359</v>
       </c>
       <c r="E53" t="n">
-        <v>0.004869039549467532</v>
+        <v>0.004884769542416435</v>
       </c>
       <c r="F53" t="n">
-        <v>0.7215904896594297</v>
+        <v>0.747327937025999</v>
       </c>
       <c r="G53" t="n">
-        <v>0.00357759049344102</v>
+        <v>0.01376937941294494</v>
       </c>
       <c r="H53" t="n">
-        <v>0.6528527229086913</v>
+        <v>0.6852618333117529</v>
       </c>
       <c r="I53" t="n">
-        <v>0.8067637572084841</v>
+        <v>0.8231616598718366</v>
       </c>
       <c r="J53" t="n">
-        <v>6.807</v>
+        <v>0.439</v>
       </c>
       <c r="K53" t="n">
-        <v>0.8912</v>
+        <v>0.9132</v>
       </c>
       <c r="L53" t="n">
-        <v>0.7288</v>
+        <v>0.7605</v>
       </c>
       <c r="M53" t="n">
-        <v>0.653</v>
+        <v>0.7102000000000001</v>
       </c>
       <c r="N53" t="n">
-        <v>0.8246</v>
+        <v>0.8185</v>
       </c>
       <c r="O53" t="n">
-        <v>0.5974</v>
+        <v>0.6513</v>
       </c>
       <c r="P53" t="n">
-        <v>0.4183</v>
+        <v>0.3624</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LogReg</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3439,43 +3439,43 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.8850131604431113</v>
+        <v>0.9057562632928381</v>
       </c>
       <c r="E54" t="n">
-        <v>0.004830727805954928</v>
+        <v>0.003212375345637456</v>
       </c>
       <c r="F54" t="n">
-        <v>0.7236380792058493</v>
+        <v>0.7493470312335072</v>
       </c>
       <c r="G54" t="n">
-        <v>0.003262651308187069</v>
+        <v>0.006349929513041751</v>
       </c>
       <c r="H54" t="n">
-        <v>0.6592766700839555</v>
+        <v>0.6980245716132399</v>
       </c>
       <c r="I54" t="n">
-        <v>0.8021871624967385</v>
+        <v>0.8090520545643567</v>
       </c>
       <c r="J54" t="n">
-        <v>6.385</v>
+        <v>3.281</v>
       </c>
       <c r="K54" t="n">
-        <v>0.8911</v>
+        <v>0.9072</v>
       </c>
       <c r="L54" t="n">
-        <v>0.731</v>
+        <v>0.7613</v>
       </c>
       <c r="M54" t="n">
-        <v>0.6581</v>
+        <v>0.7294</v>
       </c>
       <c r="N54" t="n">
-        <v>0.8221000000000001</v>
+        <v>0.7961</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6016</v>
+        <v>0.6564</v>
       </c>
       <c r="P54" t="n">
-        <v>0.4137</v>
+        <v>0.3845</v>
       </c>
     </row>
     <row r="55">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LogReg</t>
+          <t>SVM_lineal</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3495,43 +3495,43 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.8845935644281168</v>
+        <v>0.9054210519767842</v>
       </c>
       <c r="E55" t="n">
-        <v>0.004943200072061573</v>
+        <v>0.004775983310566349</v>
       </c>
       <c r="F55" t="n">
-        <v>0.7200656311241855</v>
+        <v>0.7487598873695469</v>
       </c>
       <c r="G55" t="n">
-        <v>0.009654675623845083</v>
+        <v>0.004590734269444388</v>
       </c>
       <c r="H55" t="n">
-        <v>0.7756228114556811</v>
+        <v>0.8012342359450247</v>
       </c>
       <c r="I55" t="n">
-        <v>0.6721329842618973</v>
+        <v>0.7031519018119458</v>
       </c>
       <c r="J55" t="n">
-        <v>5.926</v>
+        <v>65.28</v>
       </c>
       <c r="K55" t="n">
-        <v>0.8911</v>
+        <v>0.9109</v>
       </c>
       <c r="L55" t="n">
-        <v>0.7222</v>
+        <v>0.7524999999999999</v>
       </c>
       <c r="M55" t="n">
-        <v>0.7658</v>
+        <v>0.7963</v>
       </c>
       <c r="N55" t="n">
-        <v>0.6833</v>
+        <v>0.7133</v>
       </c>
       <c r="O55" t="n">
-        <v>0.6163999999999999</v>
+        <v>0.6579</v>
       </c>
       <c r="P55" t="n">
-        <v>0.365</v>
+        <v>0.3317</v>
       </c>
     </row>
     <row r="56">
@@ -3542,52 +3542,52 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SVM_lineal</t>
+          <t>SGDElasticNet</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.8843576981597293</v>
+        <v>0.9051599001258989</v>
       </c>
       <c r="E56" t="n">
-        <v>0.004359519374954015</v>
+        <v>0.003946958430842508</v>
       </c>
       <c r="F56" t="n">
-        <v>0.7255033237336189</v>
+        <v>0.7393836496871475</v>
       </c>
       <c r="G56" t="n">
-        <v>0.006104318062521838</v>
+        <v>0.007832908049006399</v>
       </c>
       <c r="H56" t="n">
-        <v>0.664561018718131</v>
+        <v>0.7825349652936302</v>
       </c>
       <c r="I56" t="n">
-        <v>0.7990083613971797</v>
+        <v>0.7017556429939472</v>
       </c>
       <c r="J56" t="n">
-        <v>222.988</v>
+        <v>0.445</v>
       </c>
       <c r="K56" t="n">
-        <v>0.8894</v>
+        <v>0.9069</v>
       </c>
       <c r="L56" t="n">
-        <v>0.7307</v>
+        <v>0.7494</v>
       </c>
       <c r="M56" t="n">
-        <v>0.6602</v>
+        <v>0.8022</v>
       </c>
       <c r="N56" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.7030999999999999</v>
       </c>
       <c r="O56" t="n">
-        <v>0.6018</v>
+        <v>0.6552</v>
       </c>
       <c r="P56" t="n">
-        <v>0.3695</v>
+        <v>0.3398</v>
       </c>
     </row>
     <row r="57">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LDA</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3607,155 +3607,155 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.8843329932241243</v>
+        <v>0.9038660096861791</v>
       </c>
       <c r="E57" t="n">
-        <v>0.004412754167309445</v>
+        <v>0.00580205681122376</v>
       </c>
       <c r="F57" t="n">
-        <v>0.7249502786152631</v>
+        <v>0.7359116552775953</v>
       </c>
       <c r="G57" t="n">
-        <v>0.00626459617405727</v>
+        <v>0.007200138561096124</v>
       </c>
       <c r="H57" t="n">
-        <v>0.6599831817691921</v>
+        <v>0.6491643590957055</v>
       </c>
       <c r="I57" t="n">
-        <v>0.8043477488204299</v>
+        <v>0.849860858790049</v>
       </c>
       <c r="J57" t="n">
-        <v>3.107</v>
+        <v>1.413</v>
       </c>
       <c r="K57" t="n">
-        <v>0.8898</v>
+        <v>0.9001</v>
       </c>
       <c r="L57" t="n">
-        <v>0.728</v>
+        <v>0.7337</v>
       </c>
       <c r="M57" t="n">
-        <v>0.6538</v>
+        <v>0.6777</v>
       </c>
       <c r="N57" t="n">
-        <v>0.821</v>
+        <v>0.7997</v>
       </c>
       <c r="O57" t="n">
-        <v>0.5966</v>
+        <v>0.6103</v>
       </c>
       <c r="P57" t="n">
-        <v>0.4215</v>
+        <v>0.6812</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>BernoulliNB</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.8841486780021585</v>
+        <v>0.9026765293335541</v>
       </c>
       <c r="E58" t="n">
-        <v>0.005967561688845147</v>
+        <v>0.004878767896935301</v>
       </c>
       <c r="F58" t="n">
-        <v>0.7209644616533369</v>
+        <v>0.7361697829446927</v>
       </c>
       <c r="G58" t="n">
-        <v>0.005524605109551882</v>
+        <v>0.01112601087569545</v>
       </c>
       <c r="H58" t="n">
-        <v>0.7132624744453478</v>
+        <v>0.7754078384204025</v>
       </c>
       <c r="I58" t="n">
-        <v>0.7289597892000572</v>
+        <v>0.7015024827315458</v>
       </c>
       <c r="J58" t="n">
-        <v>0.331</v>
+        <v>2.989</v>
       </c>
       <c r="K58" t="n">
-        <v>0.8875</v>
+        <v>0.9109</v>
       </c>
       <c r="L58" t="n">
-        <v>0.7239</v>
+        <v>0.7374000000000001</v>
       </c>
       <c r="M58" t="n">
-        <v>0.701</v>
+        <v>0.8228</v>
       </c>
       <c r="N58" t="n">
-        <v>0.7483</v>
+        <v>0.668</v>
       </c>
       <c r="O58" t="n">
-        <v>0.6044</v>
+        <v>0.6441</v>
       </c>
       <c r="P58" t="n">
-        <v>0.4728</v>
+        <v>0.373</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>BernoulliNB</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.8841486780021585</v>
+        <v>0.8999538184092056</v>
       </c>
       <c r="E59" t="n">
-        <v>0.005967561688845147</v>
+        <v>0.003311414395632856</v>
       </c>
       <c r="F59" t="n">
-        <v>0.7209644616533369</v>
+        <v>0.7329380126007593</v>
       </c>
       <c r="G59" t="n">
-        <v>0.005524605109551882</v>
+        <v>0.009663686372255531</v>
       </c>
       <c r="H59" t="n">
-        <v>0.7132624744453478</v>
+        <v>0.6545947385865329</v>
       </c>
       <c r="I59" t="n">
-        <v>0.7289597892000572</v>
+        <v>0.8347279496522884</v>
       </c>
       <c r="J59" t="n">
-        <v>0.286</v>
+        <v>2.478</v>
       </c>
       <c r="K59" t="n">
-        <v>0.8875</v>
+        <v>0.9133</v>
       </c>
       <c r="L59" t="n">
-        <v>0.7239</v>
+        <v>0.7453</v>
       </c>
       <c r="M59" t="n">
-        <v>0.701</v>
+        <v>0.6617</v>
       </c>
       <c r="N59" t="n">
-        <v>0.7483</v>
+        <v>0.8531</v>
       </c>
       <c r="O59" t="n">
-        <v>0.6044</v>
+        <v>0.6201</v>
       </c>
       <c r="P59" t="n">
-        <v>0.4728</v>
+        <v>0.4213</v>
       </c>
     </row>
     <row r="60">
@@ -3766,276 +3766,276 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SVM_lineal</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.8839391384077853</v>
+        <v>0.8997149781030049</v>
       </c>
       <c r="E60" t="n">
-        <v>0.00432949259336935</v>
+        <v>0.004231156829102635</v>
       </c>
       <c r="F60" t="n">
-        <v>0.7266021910022269</v>
+        <v>0.7267192283247618</v>
       </c>
       <c r="G60" t="n">
-        <v>0.005461443680121344</v>
+        <v>0.01577460752560449</v>
       </c>
       <c r="H60" t="n">
-        <v>0.6664119892739955</v>
+        <v>0.7864884931006975</v>
       </c>
       <c r="I60" t="n">
-        <v>0.7990086845117457</v>
+        <v>0.6805268544554671</v>
       </c>
       <c r="J60" t="n">
-        <v>313.818</v>
+        <v>2.677</v>
       </c>
       <c r="K60" t="n">
-        <v>0.8892</v>
+        <v>0.8977000000000001</v>
       </c>
       <c r="L60" t="n">
-        <v>0.7322</v>
+        <v>0.7271</v>
       </c>
       <c r="M60" t="n">
-        <v>0.6627</v>
+        <v>0.7665999999999999</v>
       </c>
       <c r="N60" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.6914</v>
       </c>
       <c r="O60" t="n">
-        <v>0.6042999999999999</v>
+        <v>0.6223</v>
       </c>
       <c r="P60" t="n">
-        <v>0.4181</v>
+        <v>0.7409</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>BernoulliNB</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.8834440899523732</v>
+        <v>0.8904495092967712</v>
       </c>
       <c r="E61" t="n">
-        <v>0.006091741210467352</v>
+        <v>0.0127432871352812</v>
       </c>
       <c r="F61" t="n">
-        <v>0.719159332462157</v>
+        <v>0.7261581011517647</v>
       </c>
       <c r="G61" t="n">
-        <v>0.006442997893351844</v>
+        <v>0.01875638316318416</v>
       </c>
       <c r="H61" t="n">
-        <v>0.6634652662075602</v>
+        <v>0.6575439998429703</v>
       </c>
       <c r="I61" t="n">
-        <v>0.7851511893443279</v>
+        <v>0.8189757914489345</v>
       </c>
       <c r="J61" t="n">
-        <v>2.696</v>
+        <v>2.077</v>
       </c>
       <c r="K61" t="n">
-        <v>0.8868</v>
+        <v>0.8931</v>
       </c>
       <c r="L61" t="n">
-        <v>0.7212</v>
+        <v>0.7156</v>
       </c>
       <c r="M61" t="n">
-        <v>0.6536999999999999</v>
+        <v>0.6206</v>
       </c>
       <c r="N61" t="n">
-        <v>0.8043</v>
+        <v>0.8449</v>
       </c>
       <c r="O61" t="n">
-        <v>0.5884</v>
+        <v>0.5709</v>
       </c>
       <c r="P61" t="n">
-        <v>0.5286</v>
+        <v>0.8991</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Perceptron</t>
+          <t>BernoulliNB</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.8832410336398798</v>
+        <v>0.8841486780021585</v>
       </c>
       <c r="E62" t="n">
-        <v>0.007139590517034026</v>
+        <v>0.005967561688845147</v>
       </c>
       <c r="F62" t="n">
-        <v>0.7158664191688076</v>
+        <v>0.7209644616533369</v>
       </c>
       <c r="G62" t="n">
-        <v>0.00986043738027908</v>
+        <v>0.005524605109551882</v>
       </c>
       <c r="H62" t="n">
-        <v>0.6531384758078419</v>
+        <v>0.7132624744453478</v>
       </c>
       <c r="I62" t="n">
-        <v>0.7923979220502264</v>
+        <v>0.7289597892000572</v>
       </c>
       <c r="J62" t="n">
-        <v>8.765000000000001</v>
+        <v>0.238</v>
       </c>
       <c r="K62" t="n">
-        <v>0.8915</v>
+        <v>0.8875</v>
       </c>
       <c r="L62" t="n">
-        <v>0.7274</v>
+        <v>0.7239</v>
       </c>
       <c r="M62" t="n">
-        <v>0.6519</v>
+        <v>0.701</v>
       </c>
       <c r="N62" t="n">
-        <v>0.8226</v>
+        <v>0.7483</v>
       </c>
       <c r="O62" t="n">
-        <v>0.5953000000000001</v>
+        <v>0.6044</v>
       </c>
       <c r="P62" t="n">
-        <v>0.4494</v>
+        <v>0.4728</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SVM_lineal</t>
+          <t>BernoulliNB</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.8829966625011728</v>
+        <v>0.8841486780021585</v>
       </c>
       <c r="E63" t="n">
-        <v>0.004634565943259712</v>
+        <v>0.005967561688845147</v>
       </c>
       <c r="F63" t="n">
-        <v>0.7198124238707404</v>
+        <v>0.7209644616533369</v>
       </c>
       <c r="G63" t="n">
-        <v>0.008186755279267368</v>
+        <v>0.005524605109551882</v>
       </c>
       <c r="H63" t="n">
-        <v>0.7781570502099299</v>
+        <v>0.7132624744453478</v>
       </c>
       <c r="I63" t="n">
-        <v>0.6698444445701002</v>
+        <v>0.7289597892000572</v>
       </c>
       <c r="J63" t="n">
-        <v>196.844</v>
+        <v>0.226</v>
       </c>
       <c r="K63" t="n">
-        <v>0.8898</v>
+        <v>0.8875</v>
       </c>
       <c r="L63" t="n">
-        <v>0.7236</v>
+        <v>0.7239</v>
       </c>
       <c r="M63" t="n">
-        <v>0.773</v>
+        <v>0.701</v>
       </c>
       <c r="N63" t="n">
-        <v>0.6802</v>
+        <v>0.7483</v>
       </c>
       <c r="O63" t="n">
-        <v>0.6194</v>
+        <v>0.6044</v>
       </c>
       <c r="P63" t="n">
-        <v>0.3656</v>
+        <v>0.4728</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LDA</t>
+          <t>BernoulliNB</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.8823181498223265</v>
+        <v>0.8834440899523732</v>
       </c>
       <c r="E64" t="n">
-        <v>0.004427890999659801</v>
+        <v>0.006091741210467352</v>
       </c>
       <c r="F64" t="n">
-        <v>0.714960077452233</v>
+        <v>0.719159332462157</v>
       </c>
       <c r="G64" t="n">
-        <v>0.01017420782088104</v>
+        <v>0.006442997893351844</v>
       </c>
       <c r="H64" t="n">
-        <v>0.7588041582669012</v>
+        <v>0.6634652662075602</v>
       </c>
       <c r="I64" t="n">
-        <v>0.6762009966468786</v>
+        <v>0.7851511893443279</v>
       </c>
       <c r="J64" t="n">
-        <v>4.421</v>
+        <v>1.221</v>
       </c>
       <c r="K64" t="n">
-        <v>0.8887</v>
+        <v>0.8868</v>
       </c>
       <c r="L64" t="n">
-        <v>0.726</v>
+        <v>0.7212</v>
       </c>
       <c r="M64" t="n">
-        <v>0.7599</v>
+        <v>0.6536999999999999</v>
       </c>
       <c r="N64" t="n">
-        <v>0.695</v>
+        <v>0.8043</v>
       </c>
       <c r="O64" t="n">
-        <v>0.6197</v>
+        <v>0.5884</v>
       </c>
       <c r="P64" t="n">
-        <v>0.37</v>
+        <v>0.5286</v>
       </c>
     </row>
     <row r="65">
@@ -4046,52 +4046,52 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LDA</t>
+          <t>Perceptron</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.8823181498223265</v>
+        <v>0.8832410336398798</v>
       </c>
       <c r="E65" t="n">
-        <v>0.004427890999659801</v>
+        <v>0.007139590517034026</v>
       </c>
       <c r="F65" t="n">
-        <v>0.714960077452233</v>
+        <v>0.7158664191688076</v>
       </c>
       <c r="G65" t="n">
-        <v>0.01017420782088104</v>
+        <v>0.00986043738027908</v>
       </c>
       <c r="H65" t="n">
-        <v>0.7588041582669012</v>
+        <v>0.6531384758078419</v>
       </c>
       <c r="I65" t="n">
-        <v>0.6762009966468786</v>
+        <v>0.7923979220502264</v>
       </c>
       <c r="J65" t="n">
-        <v>5.021</v>
+        <v>3.442</v>
       </c>
       <c r="K65" t="n">
-        <v>0.8887</v>
+        <v>0.8915</v>
       </c>
       <c r="L65" t="n">
-        <v>0.726</v>
+        <v>0.7274</v>
       </c>
       <c r="M65" t="n">
-        <v>0.7599</v>
+        <v>0.6519</v>
       </c>
       <c r="N65" t="n">
-        <v>0.695</v>
+        <v>0.8226</v>
       </c>
       <c r="O65" t="n">
-        <v>0.6197</v>
+        <v>0.5953000000000001</v>
       </c>
       <c r="P65" t="n">
-        <v>0.37</v>
+        <v>0.4494</v>
       </c>
     </row>
     <row r="66">
@@ -4129,7 +4129,7 @@
         <v>0.5260559585960995</v>
       </c>
       <c r="J66" t="n">
-        <v>8.106</v>
+        <v>2.642</v>
       </c>
       <c r="K66" t="n">
         <v>0.8597</v>
@@ -4185,7 +4185,7 @@
         <v>0.5100422391516304</v>
       </c>
       <c r="J67" t="n">
-        <v>5.042</v>
+        <v>2.771</v>
       </c>
       <c r="K67" t="n">
         <v>0.855</v>
@@ -4241,7 +4241,7 @@
         <v>0.7611215629697783</v>
       </c>
       <c r="J68" t="n">
-        <v>1.685</v>
+        <v>0.828</v>
       </c>
       <c r="K68" t="n">
         <v>0.8695000000000001</v>
@@ -4297,7 +4297,7 @@
         <v>0.6872589464364907</v>
       </c>
       <c r="J69" t="n">
-        <v>3.378</v>
+        <v>2.048</v>
       </c>
       <c r="K69" t="n">
         <v>0.8682</v>
@@ -4353,7 +4353,7 @@
         <v>0.6872589464364907</v>
       </c>
       <c r="J70" t="n">
-        <v>5.223</v>
+        <v>2.635</v>
       </c>
       <c r="K70" t="n">
         <v>0.8682</v>

</xml_diff>

<commit_message>
Cierre Fase 6: arquitectura C (m01a-d, m02+m02a-b, m03+m03a-b, m04+m04a-d, m05, m06)
- Reorganizacion completa Fase 6 segun auditoria Ruta B

- Nuevo notebook agregador f6_m04d_robustez_temporal (Sec 4.8 TFM)

- Navegacion HTML corregida en src/html/navegacion.py

- 17/17 notebooks ejecutados sin errores via f6_m00_ejecucion

- HTMLs regenerados con menu actualizado en todas las fases

- Limpieza de archivos _old, _BACKUP y duplicados
</commit_message>
<xml_diff>
--- a/data/05_modelado/results/resultados_maestro.xlsx
+++ b/data/05_modelado/results/resultados_maestro.xlsx
@@ -545,7 +545,7 @@
         <v>0.7935408590485407</v>
       </c>
       <c r="J2" t="n">
-        <v>4.11</v>
+        <v>5.81</v>
       </c>
       <c r="K2" t="n">
         <v>0.9573</v>
@@ -601,7 +601,7 @@
         <v>0.8611740690867409</v>
       </c>
       <c r="J3" t="n">
-        <v>4.638</v>
+        <v>5.958</v>
       </c>
       <c r="K3" t="n">
         <v>0.9572000000000001</v>
@@ -657,7 +657,7 @@
         <v>0.808414387968506</v>
       </c>
       <c r="J4" t="n">
-        <v>3.96</v>
+        <v>5.582</v>
       </c>
       <c r="K4" t="n">
         <v>0.9560999999999999</v>
@@ -713,7 +713,7 @@
         <v>0.7896000730238919</v>
       </c>
       <c r="J5" t="n">
-        <v>4.562</v>
+        <v>11.247</v>
       </c>
       <c r="K5" t="n">
         <v>0.9564</v>
@@ -769,7 +769,7 @@
         <v>0.8696920960522669</v>
       </c>
       <c r="J6" t="n">
-        <v>4.837</v>
+        <v>9.07</v>
       </c>
       <c r="K6" t="n">
         <v>0.9567</v>
@@ -825,7 +825,7 @@
         <v>0.8072708047410601</v>
       </c>
       <c r="J7" t="n">
-        <v>6.519</v>
+        <v>10.553</v>
       </c>
       <c r="K7" t="n">
         <v>0.9550999999999999</v>
@@ -993,7 +993,7 @@
         <v>0.8668948124764227</v>
       </c>
       <c r="J10" t="n">
-        <v>9.615</v>
+        <v>25.825</v>
       </c>
       <c r="K10" t="n">
         <v>0.953</v>
@@ -1049,7 +1049,7 @@
         <v>0.7753606564395522</v>
       </c>
       <c r="J11" t="n">
-        <v>10.697</v>
+        <v>25.352</v>
       </c>
       <c r="K11" t="n">
         <v>0.9536</v>
@@ -1105,7 +1105,7 @@
         <v>0.8023123693910341</v>
       </c>
       <c r="J12" t="n">
-        <v>13.366</v>
+        <v>32.373</v>
       </c>
       <c r="K12" t="n">
         <v>0.9519</v>
@@ -1665,7 +1665,7 @@
         <v>0.7677332139963536</v>
       </c>
       <c r="J22" t="n">
-        <v>19.913</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="K22" t="n">
         <v>0.9489</v>
@@ -1721,7 +1721,7 @@
         <v>0.7677332139963536</v>
       </c>
       <c r="J23" t="n">
-        <v>13.523</v>
+        <v>18.66</v>
       </c>
       <c r="K23" t="n">
         <v>0.9489</v>
@@ -1777,7 +1777,7 @@
         <v>0.8105763475291026</v>
       </c>
       <c r="J24" t="n">
-        <v>25.891</v>
+        <v>21.543</v>
       </c>
       <c r="K24" t="n">
         <v>0.947</v>

</xml_diff>